<commit_message>
Changes up to 9/16/26; Add .code-workspace file
</commit_message>
<xml_diff>
--- a/tests/test_data/col_info.xlsx
+++ b/tests/test_data/col_info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Mac\Home\Box Sync\Projects\Python_ModelingToolbox\tests\test_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15214767-3311-48F8-862C-03A38785989F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B7C396C-EFD4-4500-B50A-D961E6BEAA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1087" yWindow="1455" windowWidth="28801" windowHeight="11588" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1763" yWindow="2130" windowWidth="28800" windowHeight="11588" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cols" sheetId="5" r:id="rId1"/>
@@ -55,7 +55,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>j.d.landgrebe:</t>
         </r>
@@ -64,7 +64,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 </t>
@@ -351,14 +351,14 @@
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">

</xml_diff>